<commit_message>
improving xlsx files as Monica suggested
</commit_message>
<xml_diff>
--- a/static/results/2026_territoriale_ammessi_nazionali.xlsx
+++ b/static/results/2026_territoriale_ammessi_nazionali.xlsx
@@ -534,7 +534,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -555,6 +555,13 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -599,8 +606,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -626,7 +637,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L20"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="23.32"/>
@@ -642,41 +653,41 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="7.91"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+    <row r="1" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="0" t="s">
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="0" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="0" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
     </row>
@@ -708,7 +719,7 @@
       <c r="I2" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="K2" s="0" t="n">
@@ -746,7 +757,7 @@
       <c r="I3" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" s="2" t="s">
         <v>30</v>
       </c>
       <c r="K3" s="0" t="n">
@@ -784,7 +795,7 @@
       <c r="I4" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="J4" s="2" t="s">
         <v>40</v>
       </c>
       <c r="K4" s="0" t="n">
@@ -822,7 +833,7 @@
       <c r="I5" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="J5" s="2" t="s">
         <v>50</v>
       </c>
       <c r="K5" s="0" t="n">
@@ -860,7 +871,7 @@
       <c r="I6" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="J6" s="2" t="s">
         <v>57</v>
       </c>
       <c r="K6" s="0" t="n">
@@ -898,7 +909,7 @@
       <c r="I7" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="J7" s="2" t="s">
         <v>65</v>
       </c>
       <c r="K7" s="0" t="n">
@@ -936,7 +947,7 @@
       <c r="I8" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="J8" s="2" t="s">
         <v>69</v>
       </c>
       <c r="K8" s="0" t="n">
@@ -974,7 +985,7 @@
       <c r="I9" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="J9" s="2" t="s">
         <v>76</v>
       </c>
       <c r="K9" s="0" t="n">
@@ -1012,7 +1023,7 @@
       <c r="I10" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="J10" s="1" t="s">
+      <c r="J10" s="2" t="s">
         <v>85</v>
       </c>
       <c r="K10" s="0" t="n">
@@ -1050,7 +1061,7 @@
       <c r="I11" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="J11" s="1" t="s">
+      <c r="J11" s="2" t="s">
         <v>94</v>
       </c>
       <c r="K11" s="0" t="n">
@@ -1088,7 +1099,7 @@
       <c r="I12" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="J12" s="1" t="s">
+      <c r="J12" s="2" t="s">
         <v>103</v>
       </c>
       <c r="K12" s="0" t="n">
@@ -1126,7 +1137,7 @@
       <c r="I13" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="J13" s="1" t="s">
+      <c r="J13" s="2" t="s">
         <v>112</v>
       </c>
       <c r="K13" s="0" t="n">
@@ -1164,7 +1175,7 @@
       <c r="I14" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="J14" s="1" t="s">
+      <c r="J14" s="2" t="s">
         <v>121</v>
       </c>
       <c r="K14" s="0" t="n">
@@ -1202,7 +1213,7 @@
       <c r="I15" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="J15" s="1" t="s">
+      <c r="J15" s="2" t="s">
         <v>129</v>
       </c>
       <c r="K15" s="0" t="n">
@@ -1240,7 +1251,7 @@
       <c r="I16" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="J16" s="1" t="s">
+      <c r="J16" s="2" t="s">
         <v>136</v>
       </c>
       <c r="K16" s="0" t="n">
@@ -1278,7 +1289,7 @@
       <c r="I17" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="J17" s="1" t="s">
+      <c r="J17" s="2" t="s">
         <v>143</v>
       </c>
       <c r="K17" s="0" t="n">
@@ -1316,7 +1327,7 @@
       <c r="I18" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="J18" s="1" t="s">
+      <c r="J18" s="2" t="s">
         <v>151</v>
       </c>
       <c r="K18" s="0" t="n">
@@ -1354,7 +1365,7 @@
       <c r="I19" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="J19" s="1" t="s">
+      <c r="J19" s="2" t="s">
         <v>160</v>
       </c>
       <c r="K19" s="0" t="n">
@@ -1392,7 +1403,7 @@
       <c r="I20" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="J20" s="1" t="s">
+      <c r="J20" s="2" t="s">
         <v>167</v>
       </c>
       <c r="K20" s="0" t="n">

</xml_diff>